<commit_message>
lower-case dispensary for consistency
</commit_message>
<xml_diff>
--- a/input/Use Group Chart - Complete Use List with NAICS.xlsx
+++ b/input/Use Group Chart - Complete Use List with NAICS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m_carper\Documents\GitHub\edr-use-query-tool\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4189780-326D-4717-8CA8-6E7D51E53646}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E799DAF3-C2F1-4C6A-B462-6D2E57BF8FBC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CF69924-4D7B-49E6-ADFC-15C8E9BB2002}"/>
   </bookViews>
@@ -1831,7 +1831,7 @@
     </r>
   </si>
   <si>
-    <t>Cannabis Dispensaries*</t>
+    <t>Cannabis dispensaries*</t>
   </si>
 </sst>
 </file>
@@ -12905,7 +12905,7 @@
       </c>
       <c r="D106" s="32" t="str">
         <f t="shared" si="1"/>
-        <v>Cannabis Dispensaries*</v>
+        <v>Cannabis dispensaries*</v>
       </c>
       <c r="E106" s="37" t="e" cm="1">
         <f t="array" aca="1" ref="E106" ca="1">MID(C106,FIND("(",C106,LOOKUP(2,1/(MID(C106,ROW(INDIRECT("1:"&amp;LEN(C106))),1)="("),ROW(INDIRECT("1:"&amp;LEN(C106)))))+1,FIND(")",C106,LOOKUP(2,1/(MID(C106,ROW(INDIRECT("1:"&amp;LEN(C106))),1)="("),ROW(INDIRECT("1:"&amp;LEN(C106)))))-FIND("(",C106,LOOKUP(2,1/(MID(C106,ROW(INDIRECT("1:"&amp;LEN(C106))),1)="("),ROW(INDIRECT("1:"&amp;LEN(C106)))))-1)</f>
@@ -21790,7 +21790,7 @@
         <v>350</v>
       </c>
       <c r="D195" s="32" t="str">
-        <f t="shared" ref="D195:D245" si="3">_xlfn.TEXTAFTER(C195," - ",,,,C195)</f>
+        <f t="shared" ref="D195:D244" si="3">_xlfn.TEXTAFTER(C195," - ",,,,C195)</f>
         <v>Dead storage of motor vehicles </v>
       </c>
       <c r="E195" s="37" t="e" cm="1">

</xml_diff>

<commit_message>
revised Use Notes, removed cols from View All table
</commit_message>
<xml_diff>
--- a/input/Use Group Chart - Complete Use List with NAICS.xlsx
+++ b/input/Use Group Chart - Complete Use List with NAICS.xlsx
@@ -1,25 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m_carper\Documents\GitHub\edr-use-query-tool\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344A5CD9-62FE-44DD-A26F-92EC6579EFCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E21BE1-1486-46FA-A78C-B7461BB5E13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CF69924-4D7B-49E6-ADFC-15C8E9BB2002}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CF69924-4D7B-49E6-ADFC-15C8E9BB2002}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$D$1:$D$244</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$K$1:$K$244</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -62,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6725" uniqueCount="528">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6725" uniqueCount="530">
   <si>
     <t>Use Group</t>
   </si>
@@ -1810,19 +1809,7 @@
     <t>459210 News dealers; 459210 Newsstands (i.e., permanent); 459210 Magazine stands (i.e., permanent)</t>
   </si>
   <si>
-    <t>NAICS index assigned for tool usability, relationship not officially defined in Zoning Resolution</t>
-  </si>
-  <si>
-    <t>NAICS join not performed b/c laundry and dry cleaning not separated at NAICS index level</t>
-  </si>
-  <si>
-    <t>If court is indoors, falls into UG VI Services #Health and fitness establishments#</t>
-  </si>
-  <si>
     <t>Not an official Zoning Resolution use - added manually, follows rules of #Schools#. See Zoning Resolution glossary for details: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
-  </si>
-  <si>
-    <t>NAICS index assigned for tool usability, relationship not officially defined in Zoning Resolution; See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
   </si>
   <si>
     <t>NAICS index assigned for tool usability, relationship not officially defined in Zoning Resolution. See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
@@ -2227,12 +2214,30 @@
   <si>
     <t>See ZR Glossary for #public parking garage# and #public parking lot# definitions: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
   </si>
+  <si>
+    <t>If court is indoors, use falls into UG VI Services #Health and fitness establishments#</t>
+  </si>
+  <si>
+    <t>NAICS join not performed b/c laundry and dry cleaning not separable at NAICS index level</t>
+  </si>
+  <si>
+    <t>NAICS indices assigned for tool usability, relationship not officially defined in Zoning Resolution. See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+  </si>
+  <si>
+    <t>NAICS index assigned for tool usability, not specified in the Zoning Resolution</t>
+  </si>
+  <si>
+    <t>NAICS index assigned for tool usability, not specified in the Zoning Resolution; See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+  </si>
+  <si>
+    <t>NAICS indices assigned for tool usability, not specified in the Zoning Resolution; See ZR Glossary for use definition: https://zr.planning.nyc.gov/article-i/chapter-2#12-10</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2328,6 +2333,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2399,7 +2411,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -2521,6 +2533,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3014,7 +3029,7 @@
       <c r="I2" s="44"/>
       <c r="J2" s="37"/>
       <c r="K2" s="44" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="L2" s="26" t="s">
         <v>35</v>
@@ -3316,7 +3331,7 @@
       <c r="I5" s="37"/>
       <c r="J5" s="37"/>
       <c r="K5" s="37" t="s">
-        <v>504</v>
+        <v>524</v>
       </c>
       <c r="L5" s="26" t="s">
         <v>47</v>
@@ -3518,7 +3533,7 @@
       <c r="I7" s="37"/>
       <c r="J7" s="37"/>
       <c r="K7" s="44" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="L7" s="26" t="s">
         <v>42</v>
@@ -3720,7 +3735,7 @@
       <c r="I9" s="37"/>
       <c r="J9" s="37"/>
       <c r="K9" s="44" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
       <c r="L9" s="26" t="s">
         <v>42</v>
@@ -3820,7 +3835,7 @@
       <c r="I10" s="38"/>
       <c r="J10" s="38"/>
       <c r="K10" s="44" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="L10" s="22" t="s">
         <v>56</v>
@@ -3920,7 +3935,7 @@
       <c r="I11" s="38"/>
       <c r="J11" s="38"/>
       <c r="K11" s="44" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
       <c r="L11" s="22" t="s">
         <v>56</v>
@@ -4020,7 +4035,7 @@
       <c r="I12" s="37"/>
       <c r="J12" s="37"/>
       <c r="K12" s="44" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="L12" s="22" t="s">
         <v>56</v>
@@ -4120,7 +4135,7 @@
       <c r="I13" s="37"/>
       <c r="J13" s="37"/>
       <c r="K13" s="44" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="L13" s="22" t="s">
         <v>56</v>
@@ -4620,7 +4635,7 @@
       <c r="I18" s="37"/>
       <c r="J18" s="37"/>
       <c r="K18" s="44" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="L18" s="26" t="s">
         <v>47</v>
@@ -4722,7 +4737,7 @@
       <c r="I19" s="37"/>
       <c r="J19" s="37"/>
       <c r="K19" s="44" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="L19" s="26" t="s">
         <v>35</v>
@@ -5224,7 +5239,7 @@
       <c r="I24" s="37"/>
       <c r="J24" s="37"/>
       <c r="K24" s="44" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="L24" s="26" t="s">
         <v>42</v>
@@ -5326,7 +5341,7 @@
       <c r="I25" s="37"/>
       <c r="J25" s="37"/>
       <c r="K25" s="37" t="s">
-        <v>505</v>
+        <v>502</v>
       </c>
       <c r="L25" s="26" t="s">
         <v>42</v>
@@ -7128,7 +7143,7 @@
       <c r="I43" s="37"/>
       <c r="J43" s="37"/>
       <c r="K43" s="44" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="L43" s="26" t="s">
         <v>47</v>
@@ -9230,7 +9245,7 @@
       <c r="I64" s="37"/>
       <c r="J64" s="37"/>
       <c r="K64" s="44" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="L64" s="27" t="s">
         <v>41</v>
@@ -9732,7 +9747,7 @@
       <c r="I69" s="37"/>
       <c r="J69" s="37"/>
       <c r="K69" s="44" t="s">
-        <v>520</v>
+        <v>516</v>
       </c>
       <c r="L69" s="26" t="s">
         <v>91</v>
@@ -10034,7 +10049,7 @@
       <c r="I72" s="37"/>
       <c r="J72" s="37"/>
       <c r="K72" s="44" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
       <c r="L72" s="27" t="s">
         <v>41</v>
@@ -10236,7 +10251,7 @@
       <c r="I74" s="37"/>
       <c r="J74" s="37"/>
       <c r="K74" s="44" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
       <c r="L74" s="27" t="s">
         <v>41</v>
@@ -10338,7 +10353,7 @@
       <c r="I75" s="37"/>
       <c r="J75" s="37"/>
       <c r="K75" s="44" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
       <c r="L75" s="27" t="s">
         <v>41</v>
@@ -10846,8 +10861,8 @@
       <c r="H80" s="37"/>
       <c r="I80" s="37"/>
       <c r="J80" s="37"/>
-      <c r="K80" s="37" t="s">
-        <v>502</v>
+      <c r="K80" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L80" s="30" t="s">
         <v>166</v>
@@ -11955,8 +11970,8 @@
       <c r="J91" s="37" t="s">
         <v>459</v>
       </c>
-      <c r="K91" s="37" t="s">
-        <v>506</v>
+      <c r="K91" s="38" t="s">
+        <v>528</v>
       </c>
       <c r="L91" s="30" t="s">
         <v>166</v>
@@ -12161,8 +12176,8 @@
       <c r="H93" s="37"/>
       <c r="I93" s="37"/>
       <c r="J93" s="37"/>
-      <c r="K93" s="37" t="s">
-        <v>502</v>
+      <c r="K93" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L93" s="30" t="s">
         <v>166</v>
@@ -12870,8 +12885,8 @@
       <c r="H100" s="37"/>
       <c r="I100" s="43"/>
       <c r="J100" s="37"/>
-      <c r="K100" s="37" t="s">
-        <v>502</v>
+      <c r="K100" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L100" s="30" t="s">
         <v>166</v>
@@ -12975,8 +12990,8 @@
       <c r="H101" s="37"/>
       <c r="I101" s="43"/>
       <c r="J101" s="37"/>
-      <c r="K101" s="37" t="s">
-        <v>502</v>
+      <c r="K101" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L101" s="30" t="s">
         <v>166</v>
@@ -16409,7 +16424,7 @@
       <c r="I135" s="37"/>
       <c r="J135" s="37"/>
       <c r="K135" s="44" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
       <c r="L135" s="27" t="s">
         <v>41</v>
@@ -16510,7 +16525,7 @@
       <c r="I136" s="37"/>
       <c r="J136" s="37"/>
       <c r="K136" s="44" t="s">
-        <v>525</v>
+        <v>521</v>
       </c>
       <c r="L136" s="27" t="s">
         <v>41</v>
@@ -16914,8 +16929,8 @@
       <c r="H140" s="41"/>
       <c r="I140" s="42"/>
       <c r="J140" s="37"/>
-      <c r="K140" s="37" t="s">
-        <v>502</v>
+      <c r="K140" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L140" s="27" t="s">
         <v>41</v>
@@ -17019,8 +17034,8 @@
       <c r="H141" s="41"/>
       <c r="I141" s="42"/>
       <c r="J141" s="37"/>
-      <c r="K141" s="37" t="s">
-        <v>502</v>
+      <c r="K141" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L141" s="27" t="s">
         <v>41</v>
@@ -17227,8 +17242,8 @@
       <c r="J143" s="37" t="s">
         <v>455</v>
       </c>
-      <c r="K143" s="37" t="s">
-        <v>502</v>
+      <c r="K143" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L143" s="27" t="s">
         <v>41</v>
@@ -17335,7 +17350,7 @@
       <c r="I144" s="37"/>
       <c r="J144" s="37"/>
       <c r="K144" s="37" t="s">
-        <v>506</v>
+        <v>529</v>
       </c>
       <c r="L144" s="27" t="s">
         <v>41</v>
@@ -17442,8 +17457,8 @@
       <c r="J145" s="37" t="s">
         <v>461</v>
       </c>
-      <c r="K145" s="37" t="s">
-        <v>502</v>
+      <c r="K145" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L145" s="27" t="s">
         <v>41</v>
@@ -17547,8 +17562,8 @@
       <c r="J146" s="37" t="s">
         <v>452</v>
       </c>
-      <c r="K146" s="37" t="s">
-        <v>502</v>
+      <c r="K146" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L146" s="27" t="s">
         <v>41</v>
@@ -17652,8 +17667,8 @@
       <c r="H147" s="37"/>
       <c r="I147" s="37"/>
       <c r="J147" s="37"/>
-      <c r="K147" s="37" t="s">
-        <v>502</v>
+      <c r="K147" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L147" s="27" t="s">
         <v>41</v>
@@ -17756,7 +17771,7 @@
       <c r="I148" s="41"/>
       <c r="J148" s="41"/>
       <c r="K148" s="37" t="s">
-        <v>503</v>
+        <v>525</v>
       </c>
       <c r="L148" s="27" t="s">
         <v>41</v>
@@ -17859,7 +17874,7 @@
       <c r="I149" s="41"/>
       <c r="J149" s="41"/>
       <c r="K149" s="37" t="s">
-        <v>503</v>
+        <v>525</v>
       </c>
       <c r="L149" s="27" t="s">
         <v>41</v>
@@ -17963,8 +17978,8 @@
       <c r="H150" s="37"/>
       <c r="I150" s="37"/>
       <c r="J150" s="37"/>
-      <c r="K150" s="37" t="s">
-        <v>502</v>
+      <c r="K150" s="45" t="s">
+        <v>527</v>
       </c>
       <c r="L150" s="27" t="s">
         <v>41</v>
@@ -18474,8 +18489,8 @@
       <c r="J155" s="37" t="s">
         <v>462</v>
       </c>
-      <c r="K155" s="37" t="s">
-        <v>507</v>
+      <c r="K155" s="38" t="s">
+        <v>526</v>
       </c>
       <c r="L155" s="27" t="s">
         <v>41</v>
@@ -18579,8 +18594,8 @@
       <c r="H156" s="37"/>
       <c r="I156" s="37"/>
       <c r="J156" s="37"/>
-      <c r="K156" s="37" t="s">
-        <v>507</v>
+      <c r="K156" s="38" t="s">
+        <v>526</v>
       </c>
       <c r="L156" s="27" t="s">
         <v>41</v>
@@ -18683,7 +18698,7 @@
       <c r="I157" s="37"/>
       <c r="J157" s="37"/>
       <c r="K157" s="37" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
       <c r="L157" s="27" t="s">
         <v>41</v>
@@ -20985,7 +21000,7 @@
       <c r="I180" s="37"/>
       <c r="J180" s="37"/>
       <c r="K180" s="44" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
       <c r="L180" s="27" t="s">
         <v>41</v>
@@ -22387,7 +22402,7 @@
       <c r="I194" s="37"/>
       <c r="J194" s="37"/>
       <c r="K194" s="44" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="L194" s="27" t="s">
         <v>41</v>
@@ -22589,7 +22604,7 @@
       <c r="I196" s="37"/>
       <c r="J196" s="37"/>
       <c r="K196" s="44" t="s">
-        <v>527</v>
+        <v>523</v>
       </c>
       <c r="L196" s="27" t="s">
         <v>41</v>

</xml_diff>